<commit_message>
Created DataProvider Util for Excel Data that is used in CreateJobAPI.
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PhoenixTestData.xlsx
+++ b/src/test/resources/testData/PhoenixTestData.xlsx
@@ -3,15 +3,20 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{EF847A01-288D-48E8-8026-EF48C5C83925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/234985d93df363b6/Desktop/SDET with Jatin/JAVA MODULE/PhoenixTestAutomationFramework/src/test/resources/testData/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{80ACB509-37D0-42E6-93E9-BE3AFE5EC0A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB503531-B70D-401A-96B1-7CC95D95919C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTestData" sheetId="1" r:id="rId1"/>
+    <sheet name="CreateJobTestData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -21,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="46">
   <si>
     <t>username</t>
   </si>
@@ -36,16 +41,145 @@
   </si>
   <si>
     <t>iameng</t>
+  </si>
+  <si>
+    <t>mst_service_location_id</t>
+  </si>
+  <si>
+    <t>mst_platform_id</t>
+  </si>
+  <si>
+    <t>mst_warrenty_status_id</t>
+  </si>
+  <si>
+    <t>mst_oem_id</t>
+  </si>
+  <si>
+    <t>customer__first_name</t>
+  </si>
+  <si>
+    <t>customer__last_name</t>
+  </si>
+  <si>
+    <t>customer__mobile_number</t>
+  </si>
+  <si>
+    <t>customer__mobile_number_alt</t>
+  </si>
+  <si>
+    <t>customer__email_id</t>
+  </si>
+  <si>
+    <t>customer__email_id_alt</t>
+  </si>
+  <si>
+    <t>customer_address__flat_number</t>
+  </si>
+  <si>
+    <t>customer_address__apartment_name</t>
+  </si>
+  <si>
+    <t>customer_address__street_name</t>
+  </si>
+  <si>
+    <t>customer_address__landmark</t>
+  </si>
+  <si>
+    <t>customer_address__area</t>
+  </si>
+  <si>
+    <t>customer_address__pincode</t>
+  </si>
+  <si>
+    <t>customer_address__country</t>
+  </si>
+  <si>
+    <t>customer_address__state</t>
+  </si>
+  <si>
+    <t>customer_product__dop</t>
+  </si>
+  <si>
+    <t>customer_product__serial_number</t>
+  </si>
+  <si>
+    <t>customer_product__imei1</t>
+  </si>
+  <si>
+    <t>customer_product__imei2</t>
+  </si>
+  <si>
+    <t>customer_product__popurl</t>
+  </si>
+  <si>
+    <t>customer_product__product_id</t>
+  </si>
+  <si>
+    <t>customer_product__mst_model_id</t>
+  </si>
+  <si>
+    <t>problems__id</t>
+  </si>
+  <si>
+    <t>problems__remark</t>
+  </si>
+  <si>
+    <t>Beahan</t>
+  </si>
+  <si>
+    <t>738-946-9369</t>
+  </si>
+  <si>
+    <t>Elfrieda56@hotmail.com</t>
+  </si>
+  <si>
+    <t>c 304</t>
+  </si>
+  <si>
+    <t>Jupiter</t>
+  </si>
+  <si>
+    <t>MG road</t>
+  </si>
+  <si>
+    <t>Bangur Nagar</t>
+  </si>
+  <si>
+    <t>Goregaon West</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>2025-04-06T18:30:00.000Z</t>
+  </si>
+  <si>
+    <t>Battery Issue</t>
+  </si>
+  <si>
+    <t>Hyman</t>
+  </si>
+  <si>
+    <t>29655900001234</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -71,8 +205,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -88,6 +223,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -353,10 +492,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -364,7 +503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -372,7 +511,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -380,7 +519,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -391,4 +530,191 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0F4CA20-2B6C-4432-98DB-103EC30334EA}">
+  <dimension ref="A1:AA2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="7" max="7" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="22.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O1" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>21</v>
+      </c>
+      <c r="R1" t="s">
+        <v>22</v>
+      </c>
+      <c r="S1" t="s">
+        <v>23</v>
+      </c>
+      <c r="T1" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" t="s">
+        <v>25</v>
+      </c>
+      <c r="V1" t="s">
+        <v>26</v>
+      </c>
+      <c r="W1" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2">
+        <v>411039</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="W2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X2">
+        <v>1</v>
+      </c>
+      <c r="Y2">
+        <v>1</v>
+      </c>
+      <c r="Z2">
+        <v>1</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>